<commit_message>
test: name the Zone 1 signals of the workbooks after the curves that zone compares
</commit_message>
<xml_diff>
--- a/examples/Model/Wind/IECA2015/Excel/Producer.xlsx
+++ b/examples/Model/Wind/IECA2015/Excel/Producer.xlsx
@@ -578,10 +578,10 @@
     <t xml:space="preserve">Consigne de puissance réactive envoyée au convertisseur </t>
   </si>
   <si>
-    <t>Puissance active injectée par le convertisseur à son point de contrôle au nœud 1</t>
-  </si>
-  <si>
-    <t>Puissance réactive injectée par le convertisseur à son point de contrôle au nœud 1</t>
+    <t>Puissance active injectée par le convertisseur à son point de contrôle (nœud 1 ou 2)</t>
+  </si>
+  <si>
+    <t>Puissance réactive injectée par le convertisseur à son point de contrôle (nœud 1 ou 2)</t>
   </si>
   <si>
     <t>Courant actif direct injecté au nœud 1</t>
@@ -9572,7 +9572,7 @@
       </c>
       <c r="D4" s="170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wind_Turbine_GEN_UPuInjTerminal</t>
+          <t xml:space="preserve">Wind_Turbine_GEN_VoltageInjTerminal</t>
         </is>
       </c>
       <c r="E4" s="171"/>
@@ -9615,7 +9615,7 @@
       </c>
       <c r="D7" s="170" t="inlineStr">
         <is>
-          <t xml:space="preserve">InternalNode1_BUS_ActivePower</t>
+          <t xml:space="preserve">Wind_Turbine_GEN_ActivePowerControlledPu</t>
         </is>
       </c>
       <c r="E7" s="171"/>
@@ -9632,7 +9632,7 @@
       </c>
       <c r="D8" s="170" t="inlineStr">
         <is>
-          <t xml:space="preserve">InternalNode1_BUS_ReactivePower</t>
+          <t xml:space="preserve">Wind_Turbine_GEN_ReactivePowerControlledPu</t>
         </is>
       </c>
       <c r="E8" s="171"/>
@@ -9683,7 +9683,7 @@
       </c>
       <c r="D11" s="170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wind_Turbine_GEN_IpInjTerminal</t>
+          <t xml:space="preserve">Wind_Turbine_GEN_ActiveCurrentInjTerminal</t>
         </is>
       </c>
       <c r="E11" s="171"/>
@@ -9700,7 +9700,7 @@
       </c>
       <c r="D12" s="172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wind_Turbine_GEN_IqInjTerminal</t>
+          <t xml:space="preserve">Wind_Turbine_GEN_ReactiveCurrentInjTerminal</t>
         </is>
       </c>
       <c r="E12" s="173"/>

</xml_diff>

<commit_message>
test: give the example workbooks the signal rows of the shipped template
</commit_message>
<xml_diff>
--- a/examples/Model/Wind/IECA2015/Excel/Producer.xlsx
+++ b/examples/Model/Wind/IECA2015/Excel/Producer.xlsx
@@ -9494,7 +9494,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7803ACAA-9DA8-4463-B943-9FCE2EFA8D33}">
-  <dimension ref="A1:U32"/>
+  <dimension ref="A1:U30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" style="3" customWidth="1"/>
@@ -9640,16 +9640,16 @@
       <c r="M8" s="5"/>
     </row>
     <row r="9" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="168" t="s">
-        <v>166</v>
-      </c>
-      <c r="B9" s="169"/>
-      <c r="C9" s="76" t="s">
-        <v>167</v>
+      <c r="A9" s="166" t="s">
+        <v>169</v>
+      </c>
+      <c r="B9" s="167"/>
+      <c r="C9" s="36" t="s">
+        <v>170</v>
       </c>
       <c r="D9" s="170" t="inlineStr">
         <is>
-          <t xml:space="preserve">InternalNode1_BUS_ActiveCurrent</t>
+          <t xml:space="preserve">Wind_Turbine_GEN_ActiveCurrentInjTerminal</t>
         </is>
       </c>
       <c r="E9" s="171"/>
@@ -9657,74 +9657,83 @@
       <c r="M9" s="5"/>
     </row>
     <row r="10" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="168" t="s">
-        <v>168</v>
-      </c>
-      <c r="B10" s="169"/>
-      <c r="C10" s="77" t="s">
-        <v>167</v>
-      </c>
-      <c r="D10" s="170" t="inlineStr">
-        <is>
-          <t xml:space="preserve">InternalNode1_BUS_ReactiveCurrent</t>
-        </is>
-      </c>
-      <c r="E10" s="171"/>
-      <c r="F10" s="5"/>
-      <c r="M10" s="5"/>
-    </row>
-    <row r="11" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="166" t="s">
-        <v>169</v>
-      </c>
-      <c r="B11" s="167"/>
-      <c r="C11" s="36" t="s">
+      <c r="A10" s="174" t="s">
+        <v>171</v>
+      </c>
+      <c r="B10" s="175"/>
+      <c r="C10" s="41" t="s">
         <v>170</v>
       </c>
-      <c r="D11" s="170" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Wind_Turbine_GEN_ActiveCurrentInjTerminal</t>
-        </is>
-      </c>
-      <c r="E11" s="171"/>
-      <c r="F11" s="5"/>
-      <c r="M11" s="5"/>
-    </row>
-    <row r="12" spans="1:21" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="174" t="s">
-        <v>171</v>
-      </c>
-      <c r="B12" s="175"/>
-      <c r="C12" s="41" t="s">
-        <v>170</v>
-      </c>
-      <c r="D12" s="172" t="inlineStr">
+      <c r="D10" s="172" t="inlineStr">
         <is>
           <t xml:space="preserve">Wind_Turbine_GEN_ReactiveCurrentInjTerminal</t>
         </is>
       </c>
-      <c r="E12" s="173"/>
-      <c r="F12" s="5"/>
+      <c r="E10" s="173"/>
+      <c r="F10" s="5"/>
+      <c r="M10" s="5"/>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="2"/>
+      <c r="M11" s="5"/>
+    </row>
+    <row r="12" spans="1:21" ht="29.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="50"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="55" t="s">
+        <v>172</v>
+      </c>
       <c r="M12" s="5"/>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="2"/>
+      <c r="N12" s="5"/>
+      <c r="O12" s="5"/>
+      <c r="P12" s="5"/>
+      <c r="Q12" s="5"/>
+      <c r="R12" s="5"/>
+      <c r="S12" s="5"/>
+      <c r="T12" s="5"/>
+      <c r="U12" s="5"/>
+    </row>
+    <row r="13" spans="1:21" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">../ReferenceCurves/Producer</t>
+        </is>
+      </c>
+      <c r="I13" s="9"/>
+      <c r="J13" s="6"/>
+      <c r="K13" s="6"/>
+      <c r="L13" s="6"/>
       <c r="M13" s="5"/>
-    </row>
-    <row r="14" spans="1:21" ht="29.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
+      <c r="P13" s="5"/>
+      <c r="Q13" s="5"/>
+      <c r="R13" s="5"/>
+      <c r="S13" s="5"/>
+      <c r="T13" s="5"/>
+      <c r="U13" s="5"/>
+    </row>
+    <row r="14" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="50"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="55" t="s">
-        <v>172</v>
-      </c>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="125"/>
+      <c r="J14" s="1"/>
+      <c r="K14" s="1"/>
+      <c r="L14" s="2"/>
       <c r="M14" s="5"/>
       <c r="N14" s="5"/>
       <c r="O14" s="5"/>
@@ -9735,16 +9744,21 @@
       <c r="T14" s="5"/>
       <c r="U14" s="5"/>
     </row>
-    <row r="15" spans="1:21" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">../ReferenceCurves/Producer</t>
-        </is>
-      </c>
-      <c r="I15" s="9"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
+    <row r="15" spans="1:21" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="150" t="s">
+        <v>174</v>
+      </c>
+      <c r="B15" s="151"/>
+      <c r="C15" s="151"/>
+      <c r="D15" s="151"/>
+      <c r="E15" s="151"/>
+      <c r="F15" s="151"/>
+      <c r="G15" s="152"/>
+      <c r="H15" s="185"/>
+      <c r="I15" s="186"/>
+      <c r="J15" s="187"/>
+      <c r="K15" s="156"/>
+      <c r="L15" s="5"/>
       <c r="M15" s="5"/>
       <c r="N15" s="5"/>
       <c r="O15" s="5"/>
@@ -9755,19 +9769,25 @@
       <c r="T15" s="5"/>
       <c r="U15" s="5"/>
     </row>
-    <row r="16" spans="1:21" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="50"/>
-      <c r="E16" s="1"/>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="125"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="2"/>
+    <row r="16" spans="1:21" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="126"/>
+      <c r="B16" s="127"/>
+      <c r="C16" s="176" t="s">
+        <v>175</v>
+      </c>
+      <c r="D16" s="157"/>
+      <c r="E16" s="157"/>
+      <c r="F16" s="157"/>
+      <c r="G16" s="128" t="s">
+        <v>176</v>
+      </c>
+      <c r="H16" s="177" t="s">
+        <v>617</v>
+      </c>
+      <c r="I16" s="178"/>
+      <c r="J16" s="178"/>
+      <c r="K16" s="179"/>
+      <c r="L16" s="5"/>
       <c r="M16" s="5"/>
       <c r="N16" s="5"/>
       <c r="O16" s="5"/>
@@ -9778,20 +9798,38 @@
       <c r="T16" s="5"/>
       <c r="U16" s="5"/>
     </row>
-    <row r="17" spans="1:21" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="150" t="s">
-        <v>174</v>
-      </c>
-      <c r="B17" s="151"/>
-      <c r="C17" s="151"/>
-      <c r="D17" s="151"/>
-      <c r="E17" s="151"/>
-      <c r="F17" s="151"/>
-      <c r="G17" s="152"/>
-      <c r="H17" s="185"/>
-      <c r="I17" s="186"/>
-      <c r="J17" s="187"/>
-      <c r="K17" s="156"/>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A17" s="53" t="s">
+        <v>177</v>
+      </c>
+      <c r="B17" s="43" t="s">
+        <v>178</v>
+      </c>
+      <c r="C17" s="65" t="s">
+        <v>179</v>
+      </c>
+      <c r="D17" s="65" t="s">
+        <v>180</v>
+      </c>
+      <c r="E17" s="65" t="s">
+        <v>181</v>
+      </c>
+      <c r="F17" s="69" t="s">
+        <v>182</v>
+      </c>
+      <c r="G17" s="54"/>
+      <c r="H17" s="65" t="s">
+        <v>618</v>
+      </c>
+      <c r="I17" s="65" t="s">
+        <v>619</v>
+      </c>
+      <c r="J17" s="65" t="s">
+        <v>620</v>
+      </c>
+      <c r="K17" s="121" t="s">
+        <v>621</v>
+      </c>
       <c r="L17" s="5"/>
       <c r="M17" s="5"/>
       <c r="N17" s="5"/>
@@ -9803,24 +9841,44 @@
       <c r="T17" s="5"/>
       <c r="U17" s="5"/>
     </row>
-    <row r="18" spans="1:21" ht="33.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="126"/>
-      <c r="B18" s="127"/>
-      <c r="C18" s="176" t="s">
-        <v>175</v>
-      </c>
-      <c r="D18" s="157"/>
-      <c r="E18" s="157"/>
-      <c r="F18" s="157"/>
-      <c r="G18" s="128" t="s">
-        <v>176</v>
-      </c>
-      <c r="H18" s="177" t="s">
-        <v>617</v>
-      </c>
-      <c r="I18" s="178"/>
-      <c r="J18" s="178"/>
-      <c r="K18" s="179"/>
+    <row r="18" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="45">
+        <v>6</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="C18" s="66" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="66" t="s">
+        <v>184</v>
+      </c>
+      <c r="E18" s="66">
+        <v>0</v>
+      </c>
+      <c r="F18" s="70">
+        <v>3</v>
+      </c>
+      <c r="G18" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.TransientBoltedSCR3.csv</t>
+        </is>
+      </c>
+      <c r="H18" s="66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non</t>
+        </is>
+      </c>
+      <c r="I18" s="66">
+        <v>30.0</v>
+      </c>
+      <c r="J18" s="66">
+        <v>0.150</v>
+      </c>
+      <c r="K18" s="122">
+        <v>15</v>
+      </c>
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
       <c r="N18" s="5"/>
@@ -9832,37 +9890,43 @@
       <c r="T18" s="5"/>
       <c r="U18" s="5"/>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A19" s="53" t="s">
-        <v>177</v>
-      </c>
-      <c r="B19" s="43" t="s">
-        <v>178</v>
-      </c>
-      <c r="C19" s="65" t="s">
-        <v>179</v>
-      </c>
-      <c r="D19" s="65" t="s">
-        <v>180</v>
-      </c>
-      <c r="E19" s="65" t="s">
-        <v>181</v>
-      </c>
-      <c r="F19" s="69" t="s">
-        <v>182</v>
-      </c>
-      <c r="G19" s="54"/>
-      <c r="H19" s="65" t="s">
-        <v>618</v>
-      </c>
-      <c r="I19" s="65" t="s">
-        <v>619</v>
-      </c>
-      <c r="J19" s="65" t="s">
-        <v>620</v>
-      </c>
-      <c r="K19" s="121" t="s">
-        <v>621</v>
+    <row r="19" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="45">
+        <v>7</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="C19" s="66" t="s">
+        <v>25</v>
+      </c>
+      <c r="D19" s="66" t="s">
+        <v>184</v>
+      </c>
+      <c r="E19" s="66">
+        <v>0</v>
+      </c>
+      <c r="F19" s="70">
+        <v>10</v>
+      </c>
+      <c r="G19" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.TransientBoltedSCR10.csv</t>
+        </is>
+      </c>
+      <c r="H19" s="66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non</t>
+        </is>
+      </c>
+      <c r="I19" s="66">
+        <v>30.0</v>
+      </c>
+      <c r="J19" s="66">
+        <v>0.150</v>
+      </c>
+      <c r="K19" s="122">
+        <v>15</v>
       </c>
       <c r="L19" s="5"/>
       <c r="M19" s="5"/>
@@ -9877,7 +9941,7 @@
     </row>
     <row r="20" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="45">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B20" s="10" t="s">
         <v>183</v>
@@ -9888,15 +9952,15 @@
       <c r="D20" s="66" t="s">
         <v>184</v>
       </c>
-      <c r="E20" s="66">
-        <v>0</v>
+      <c r="E20" s="66" t="s">
+        <v>49</v>
       </c>
       <c r="F20" s="70">
         <v>3</v>
       </c>
       <c r="G20" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.TransientBoltedSCR3.csv</t>
+          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.TransientBoltedSCR3Qmin.csv</t>
         </is>
       </c>
       <c r="H20" s="66" t="inlineStr">
@@ -9924,12 +9988,12 @@
       <c r="T20" s="5"/>
       <c r="U20" s="5"/>
     </row>
-    <row r="21" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="45">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C21" s="66" t="s">
         <v>25</v>
@@ -9941,11 +10005,11 @@
         <v>0</v>
       </c>
       <c r="F21" s="70">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G21" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.TransientBoltedSCR10.csv</t>
+          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.TransientHiZTc800.csv</t>
         </is>
       </c>
       <c r="H21" s="66" t="inlineStr">
@@ -9957,7 +10021,7 @@
         <v>30.0</v>
       </c>
       <c r="J21" s="66">
-        <v>0.150</v>
+        <v>0.8</v>
       </c>
       <c r="K21" s="122">
         <v>15</v>
@@ -9973,12 +10037,12 @@
       <c r="T21" s="5"/>
       <c r="U21" s="5"/>
     </row>
-    <row r="22" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="45">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="C22" s="66" t="s">
         <v>25</v>
@@ -9986,15 +10050,15 @@
       <c r="D22" s="66" t="s">
         <v>184</v>
       </c>
-      <c r="E22" s="66" t="s">
-        <v>49</v>
+      <c r="E22" s="66">
+        <v>0</v>
       </c>
       <c r="F22" s="70">
         <v>3</v>
       </c>
       <c r="G22" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.TransientBoltedSCR3Qmin.csv</t>
+          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.TransientHiZTc500.csv</t>
         </is>
       </c>
       <c r="H22" s="66" t="inlineStr">
@@ -10006,7 +10070,7 @@
         <v>30.0</v>
       </c>
       <c r="J22" s="66">
-        <v>0.150</v>
+        <v>0.5</v>
       </c>
       <c r="K22" s="122">
         <v>15</v>
@@ -10022,12 +10086,12 @@
       <c r="T22" s="5"/>
       <c r="U22" s="5"/>
     </row>
-    <row r="23" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="45">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C23" s="66" t="s">
         <v>25</v>
@@ -10035,15 +10099,15 @@
       <c r="D23" s="66" t="s">
         <v>184</v>
       </c>
-      <c r="E23" s="66">
-        <v>0</v>
+      <c r="E23" s="66" t="s">
+        <v>49</v>
       </c>
       <c r="F23" s="70">
         <v>3</v>
       </c>
       <c r="G23" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.TransientHiZTc800.csv</t>
+          <t xml:space="preserve">PCS_RTE-I16z1.SetPointStep.Active.csv</t>
         </is>
       </c>
       <c r="H23" s="66" t="inlineStr">
@@ -10052,10 +10116,10 @@
         </is>
       </c>
       <c r="I23" s="66">
-        <v>30.0</v>
+        <v>20.0</v>
       </c>
       <c r="J23" s="66">
-        <v>0.8</v>
+        <v>0.0</v>
       </c>
       <c r="K23" s="122">
         <v>15</v>
@@ -10071,45 +10135,33 @@
       <c r="T23" s="5"/>
       <c r="U23" s="5"/>
     </row>
-    <row r="24" spans="1:21" ht="45" x14ac:dyDescent="0.25">
-      <c r="A24" s="45">
-        <v>10</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="C24" s="66" t="s">
+    <row r="24" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="46">
+        <v>14</v>
+      </c>
+      <c r="B24" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="C24" s="73" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="66" t="s">
+      <c r="D24" s="67" t="s">
         <v>184</v>
       </c>
-      <c r="E24" s="66">
+      <c r="E24" s="67">
         <v>0</v>
       </c>
-      <c r="F24" s="70">
+      <c r="F24" s="71">
         <v>3</v>
       </c>
-      <c r="G24" s="51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.TransientHiZTc500.csv</t>
-        </is>
-      </c>
-      <c r="H24" s="66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Non</t>
-        </is>
-      </c>
-      <c r="I24" s="66">
-        <v>30.0</v>
-      </c>
-      <c r="J24" s="66">
-        <v>0.5</v>
-      </c>
-      <c r="K24" s="122">
-        <v>15</v>
-      </c>
-      <c r="L24" s="5"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="73"/>
+      <c r="I24" s="67"/>
+      <c r="J24" s="67"/>
+      <c r="K24" s="123"/>
+      <c r="L24" s="18" t="s">
+        <v>189</v>
+      </c>
       <c r="M24" s="5"/>
       <c r="N24" s="5"/>
       <c r="O24" s="5"/>
@@ -10122,10 +10174,10 @@
     </row>
     <row r="25" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="45">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C25" s="66" t="s">
         <v>25</v>
@@ -10133,15 +10185,15 @@
       <c r="D25" s="66" t="s">
         <v>184</v>
       </c>
-      <c r="E25" s="66" t="s">
-        <v>49</v>
+      <c r="E25" s="66">
+        <v>0</v>
       </c>
       <c r="F25" s="70">
         <v>3</v>
       </c>
       <c r="G25" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">PCS_RTE-I16z1.SetPointStep.Active.csv</t>
+          <t xml:space="preserve">PCS_RTE-I16z1.SetPointStep.Voltage.csv</t>
         </is>
       </c>
       <c r="H25" s="66" t="inlineStr">
@@ -10159,75 +10211,69 @@
         <v>15</v>
       </c>
       <c r="L25" s="5"/>
-      <c r="M25" s="5"/>
-      <c r="N25" s="5"/>
-      <c r="O25" s="5"/>
-      <c r="P25" s="5"/>
-      <c r="Q25" s="5"/>
-      <c r="R25" s="5"/>
-      <c r="S25" s="5"/>
-      <c r="T25" s="5"/>
-      <c r="U25" s="5"/>
-    </row>
-    <row r="26" spans="1:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="46">
-        <v>14</v>
-      </c>
-      <c r="B26" s="15" t="s">
-        <v>188</v>
-      </c>
-      <c r="C26" s="73" t="s">
+    </row>
+    <row r="26" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+      <c r="A26" s="45">
+        <v>16</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="C26" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="D26" s="67" t="s">
+      <c r="D26" s="66" t="s">
         <v>184</v>
       </c>
-      <c r="E26" s="67">
+      <c r="E26" s="66">
         <v>0</v>
       </c>
-      <c r="F26" s="71">
+      <c r="F26" s="70">
         <v>3</v>
       </c>
-      <c r="G26" s="16"/>
-      <c r="H26" s="73"/>
-      <c r="I26" s="67"/>
-      <c r="J26" s="67"/>
-      <c r="K26" s="123"/>
-      <c r="L26" s="18" t="s">
-        <v>189</v>
-      </c>
-      <c r="M26" s="5"/>
-      <c r="N26" s="5"/>
-      <c r="O26" s="5"/>
-      <c r="P26" s="5"/>
-      <c r="Q26" s="5"/>
-      <c r="R26" s="5"/>
-      <c r="S26" s="5"/>
-      <c r="T26" s="5"/>
-      <c r="U26" s="5"/>
+      <c r="G26" s="51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PCS_RTE-I16z1.SetPointStep.Reactive.csv</t>
+        </is>
+      </c>
+      <c r="H26" s="66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Non</t>
+        </is>
+      </c>
+      <c r="I26" s="66">
+        <v>20.0</v>
+      </c>
+      <c r="J26" s="66">
+        <v>0.0</v>
+      </c>
+      <c r="K26" s="122">
+        <v>15</v>
+      </c>
+      <c r="L26" s="5"/>
     </row>
     <row r="27" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="45">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C27" s="66" t="s">
-        <v>25</v>
+        <v>193</v>
       </c>
       <c r="D27" s="66" t="s">
-        <v>184</v>
-      </c>
-      <c r="E27" s="66">
-        <v>0</v>
+        <v>194</v>
+      </c>
+      <c r="E27" s="66" t="s">
+        <v>49</v>
       </c>
       <c r="F27" s="70">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G27" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">PCS_RTE-I16z1.SetPointStep.Voltage.csv</t>
+          <t xml:space="preserve">PCS_RTE-I16z1.GridVoltageStep.Rise.csv</t>
         </is>
       </c>
       <c r="H27" s="66" t="inlineStr">
@@ -10236,7 +10282,7 @@
         </is>
       </c>
       <c r="I27" s="66">
-        <v>20.0</v>
+        <v>30.0</v>
       </c>
       <c r="J27" s="66">
         <v>0.0</v>
@@ -10246,28 +10292,28 @@
       </c>
       <c r="L27" s="5"/>
     </row>
-    <row r="28" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="45">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="C28" s="66" t="s">
-        <v>25</v>
+        <v>196</v>
       </c>
       <c r="D28" s="66" t="s">
-        <v>184</v>
-      </c>
-      <c r="E28" s="66">
-        <v>0</v>
+        <v>194</v>
+      </c>
+      <c r="E28" s="66" t="s">
+        <v>45</v>
       </c>
       <c r="F28" s="70">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G28" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">PCS_RTE-I16z1.SetPointStep.Reactive.csv</t>
+          <t xml:space="preserve">PCS_RTE-I16z1.GridVoltageStep.Drop.csv</t>
         </is>
       </c>
       <c r="H28" s="66" t="inlineStr">
@@ -10276,7 +10322,7 @@
         </is>
       </c>
       <c r="I28" s="66">
-        <v>20.0</v>
+        <v>30.0</v>
       </c>
       <c r="J28" s="66">
         <v>0.0</v>
@@ -10286,28 +10332,28 @@
       </c>
       <c r="L28" s="5"/>
     </row>
-    <row r="29" spans="1:21" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="45">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="C29" s="66" t="s">
-        <v>193</v>
+        <v>25</v>
       </c>
       <c r="D29" s="66" t="s">
-        <v>194</v>
-      </c>
-      <c r="E29" s="66" t="s">
-        <v>49</v>
+        <v>184</v>
+      </c>
+      <c r="E29" s="66">
+        <v>0</v>
       </c>
       <c r="F29" s="70">
         <v>10</v>
       </c>
       <c r="G29" s="51" t="inlineStr">
         <is>
-          <t xml:space="preserve">PCS_RTE-I16z1.GridVoltageStep.Rise.csv</t>
+          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.PermanentHiZ.csv</t>
         </is>
       </c>
       <c r="H29" s="66" t="inlineStr">
@@ -10326,136 +10372,56 @@
       </c>
       <c r="L29" s="5"/>
     </row>
-    <row r="30" spans="1:21" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="45">
-        <v>18</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="C30" s="66" t="s">
-        <v>196</v>
-      </c>
-      <c r="D30" s="66" t="s">
-        <v>194</v>
-      </c>
-      <c r="E30" s="66" t="s">
-        <v>45</v>
-      </c>
-      <c r="F30" s="70">
+    <row r="30" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="47">
+        <v>24</v>
+      </c>
+      <c r="B30" s="48" t="s">
+        <v>198</v>
+      </c>
+      <c r="C30" s="68" t="s">
+        <v>25</v>
+      </c>
+      <c r="D30" s="68" t="s">
+        <v>184</v>
+      </c>
+      <c r="E30" s="68">
+        <v>0</v>
+      </c>
+      <c r="F30" s="72">
         <v>10</v>
       </c>
-      <c r="G30" s="51" t="inlineStr">
+      <c r="G30" s="52" t="inlineStr">
         <is>
-          <t xml:space="preserve">PCS_RTE-I16z1.GridVoltageStep.Drop.csv</t>
+          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.PermanentBolted.csv</t>
         </is>
       </c>
-      <c r="H30" s="66" t="inlineStr">
+      <c r="H30" s="68" t="inlineStr">
         <is>
           <t xml:space="preserve">Non</t>
         </is>
       </c>
-      <c r="I30" s="66">
+      <c r="I30" s="68">
         <v>30.0</v>
       </c>
-      <c r="J30" s="66">
+      <c r="J30" s="68">
         <v>0.0</v>
       </c>
-      <c r="K30" s="122">
+      <c r="K30" s="124">
         <v>15</v>
       </c>
       <c r="L30" s="5"/>
     </row>
-    <row r="31" spans="1:21" ht="45" x14ac:dyDescent="0.25">
-      <c r="A31" s="45">
-        <v>23</v>
-      </c>
-      <c r="B31" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="C31" s="66" t="s">
-        <v>25</v>
-      </c>
-      <c r="D31" s="66" t="s">
-        <v>184</v>
-      </c>
-      <c r="E31" s="66">
-        <v>0</v>
-      </c>
-      <c r="F31" s="70">
-        <v>10</v>
-      </c>
-      <c r="G31" s="51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.PermanentHiZ.csv</t>
-        </is>
-      </c>
-      <c r="H31" s="66" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Non</t>
-        </is>
-      </c>
-      <c r="I31" s="66">
-        <v>30.0</v>
-      </c>
-      <c r="J31" s="66">
-        <v>0.0</v>
-      </c>
-      <c r="K31" s="122">
-        <v>15</v>
-      </c>
-      <c r="L31" s="5"/>
-    </row>
-    <row r="32" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="47">
-        <v>24</v>
-      </c>
-      <c r="B32" s="48" t="s">
-        <v>198</v>
-      </c>
-      <c r="C32" s="68" t="s">
-        <v>25</v>
-      </c>
-      <c r="D32" s="68" t="s">
-        <v>184</v>
-      </c>
-      <c r="E32" s="68">
-        <v>0</v>
-      </c>
-      <c r="F32" s="72">
-        <v>10</v>
-      </c>
-      <c r="G32" s="52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PCS_RTE-I16z1.ThreePhaseFault.PermanentBolted.csv</t>
-        </is>
-      </c>
-      <c r="H32" s="68" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Non</t>
-        </is>
-      </c>
-      <c r="I32" s="68">
-        <v>30.0</v>
-      </c>
-      <c r="J32" s="68">
-        <v>0.0</v>
-      </c>
-      <c r="K32" s="124">
-        <v>15</v>
-      </c>
-      <c r="L32" s="5"/>
-    </row>
   </sheetData>
-  <mergeCells count="27">
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="H18:K18"/>
+  <mergeCells count="23">
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="H16:K16"/>
     <mergeCell ref="J2:K2"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A15:K15"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="D3:E3"/>
     <mergeCell ref="D4:E4"/>
@@ -10463,18 +10429,14 @@
     <mergeCell ref="D6:E6"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="D10:E10"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="D10:E10"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
test: declare the Zone 1 setpoints in the example dictionaries and workbooks
</commit_message>
<xml_diff>
--- a/examples/Model/Wind/IECA2015/Excel/Producer.xlsx
+++ b/examples/Model/Wind/IECA2015/Excel/Producer.xlsx
@@ -9587,7 +9587,11 @@
       <c r="C5" s="36" t="s">
         <v>162</v>
       </c>
-      <c r="D5" s="170"/>
+      <c r="D5" s="170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wind_Turbine_GEN_ActivePowerSetpointPu</t>
+        </is>
+      </c>
       <c r="E5" s="171"/>
       <c r="F5" s="5"/>
       <c r="M5" s="5"/>
@@ -9600,7 +9604,11 @@
       <c r="C6" s="36" t="s">
         <v>162</v>
       </c>
-      <c r="D6" s="170"/>
+      <c r="D6" s="170" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Wind_Turbine_GEN_ReactivePowerSetpointPu</t>
+        </is>
+      </c>
       <c r="E6" s="171"/>
       <c r="F6" s="5"/>
       <c r="M6" s="5"/>

</xml_diff>

<commit_message>
fix(examples): declare the IEC reactive capability and bound the plant reference
</commit_message>
<xml_diff>
--- a/examples/Model/Wind/IECA2015/Excel/Producer.xlsx
+++ b/examples/Model/Wind/IECA2015/Excel/Producer.xlsx
@@ -9109,7 +9109,7 @@
         <v>93</v>
       </c>
       <c r="D19" s="21">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="E19" s="21" t="s">
         <v>47</v>
@@ -9127,7 +9127,7 @@
         <v>96</v>
       </c>
       <c r="D20" s="21">
-        <v>-40</v>
+        <v>-35</v>
       </c>
       <c r="E20" s="21" t="s">
         <v>47</v>
@@ -12256,7 +12256,7 @@
         <v>383</v>
       </c>
       <c r="L10" s="103">
-        <v>999</v>
+        <v>1.1</v>
       </c>
       <c r="M10" s="100" t="s">
         <v>383</v>
@@ -12304,7 +12304,7 @@
         <v>386</v>
       </c>
       <c r="L11" s="103">
-        <v>-999</v>
+        <v>-0.8</v>
       </c>
       <c r="M11" s="100" t="s">
         <v>386</v>

</xml_diff>

<commit_message>
fix(examples): split the IEC 2020 plant communication lead-lag
</commit_message>
<xml_diff>
--- a/examples/Model/Wind/IECA2015/Excel/Producer.xlsx
+++ b/examples/Model/Wind/IECA2015/Excel/Producer.xlsx
@@ -52,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1991" uniqueCount="793">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2019" uniqueCount="805">
   <si>
     <t>format_version</t>
   </si>
@@ -2472,6 +2472,42 @@
   </si>
   <si>
     <t>false</t>
+  </si>
+  <si>
+    <t>tLagM</t>
+  </si>
+  <si>
+    <t>Communication lag time constant for PPC measurements in s</t>
+  </si>
+  <si>
+    <t>tLeadM</t>
+  </si>
+  <si>
+    <t>Communication lead time constant for PPC measurements in s</t>
+  </si>
+  <si>
+    <t>tLagPD</t>
+  </si>
+  <si>
+    <t>Communication lag time constant for PPC setpoints in s</t>
+  </si>
+  <si>
+    <t>tLeadPD</t>
+  </si>
+  <si>
+    <t>Communication lead time constant for PPC setpoints in s</t>
+  </si>
+  <si>
+    <t>tLagRef</t>
+  </si>
+  <si>
+    <t>Communication lag time constant for PPC references in s</t>
+  </si>
+  <si>
+    <t>tLeadRef</t>
+  </si>
+  <si>
+    <t>Communication lead time constant for PPC references in s</t>
   </si>
 </sst>
 </file>
@@ -5600,14 +5636,14 @@
         <v>382</v>
       </c>
       <c r="M5" s="97" t="s">
-        <v>426</v>
+        <v>793</v>
       </c>
       <c r="N5" s="100"/>
       <c r="O5" s="97" t="s">
         <v>330</v>
       </c>
       <c r="P5" s="103" t="s">
-        <v>427</v>
+        <v>794</v>
       </c>
       <c r="Q5" s="106" t="s">
         <v>394</v>
@@ -5641,29 +5677,29 @@
         <v>18</v>
       </c>
       <c r="I6" s="113"/>
-      <c r="K6" s="99" t="s">
-        <v>382</v>
-      </c>
-      <c r="L6" s="99" t="s">
-        <v>382</v>
-      </c>
-      <c r="M6" s="99" t="s">
-        <v>430</v>
-      </c>
-      <c r="N6" s="102"/>
-      <c r="O6" s="99" t="s">
-        <v>330</v>
-      </c>
-      <c r="P6" s="105" t="s">
-        <v>431</v>
-      </c>
-      <c r="Q6" s="110" t="s">
+      <c r="K6" s="98" t="s">
+        <v>382</v>
+      </c>
+      <c r="L6" s="98" t="s">
+        <v>382</v>
+      </c>
+      <c r="M6" s="98" t="s">
+        <v>795</v>
+      </c>
+      <c r="N6" s="101"/>
+      <c r="O6" s="98" t="s">
+        <v>330</v>
+      </c>
+      <c r="P6" s="104" t="s">
+        <v>796</v>
+      </c>
+      <c r="Q6" s="108" t="s">
         <v>394</v>
       </c>
-      <c r="R6" s="111" t="s">
+      <c r="R6" s="109" t="s">
         <v>18</v>
       </c>
-      <c r="S6" s="114"/>
+      <c r="S6" s="113"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="98" t="s">
@@ -5689,6 +5725,29 @@
         <v>18</v>
       </c>
       <c r="I7" s="113"/>
+      <c r="K7" s="98" t="s">
+        <v>382</v>
+      </c>
+      <c r="L7" s="98" t="s">
+        <v>382</v>
+      </c>
+      <c r="M7" s="98" t="s">
+        <v>797</v>
+      </c>
+      <c r="N7" s="101"/>
+      <c r="O7" s="98" t="s">
+        <v>330</v>
+      </c>
+      <c r="P7" s="104" t="s">
+        <v>798</v>
+      </c>
+      <c r="Q7" s="108" t="s">
+        <v>394</v>
+      </c>
+      <c r="R7" s="109" t="s">
+        <v>18</v>
+      </c>
+      <c r="S7" s="113"/>
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="98" t="s">
@@ -5714,6 +5773,29 @@
         <v>18</v>
       </c>
       <c r="I8" s="113"/>
+      <c r="K8" s="98" t="s">
+        <v>382</v>
+      </c>
+      <c r="L8" s="98" t="s">
+        <v>382</v>
+      </c>
+      <c r="M8" s="98" t="s">
+        <v>799</v>
+      </c>
+      <c r="N8" s="101"/>
+      <c r="O8" s="98" t="s">
+        <v>330</v>
+      </c>
+      <c r="P8" s="104" t="s">
+        <v>800</v>
+      </c>
+      <c r="Q8" s="108" t="s">
+        <v>394</v>
+      </c>
+      <c r="R8" s="109" t="s">
+        <v>18</v>
+      </c>
+      <c r="S8" s="113"/>
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="98" t="s">
@@ -5739,6 +5821,29 @@
         <v>18</v>
       </c>
       <c r="I9" s="113"/>
+      <c r="K9" s="98" t="s">
+        <v>382</v>
+      </c>
+      <c r="L9" s="98" t="s">
+        <v>382</v>
+      </c>
+      <c r="M9" s="98" t="s">
+        <v>801</v>
+      </c>
+      <c r="N9" s="101"/>
+      <c r="O9" s="98" t="s">
+        <v>330</v>
+      </c>
+      <c r="P9" s="104" t="s">
+        <v>802</v>
+      </c>
+      <c r="Q9" s="108" t="s">
+        <v>394</v>
+      </c>
+      <c r="R9" s="109" t="s">
+        <v>18</v>
+      </c>
+      <c r="S9" s="113"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="99" t="s">
@@ -5764,6 +5869,29 @@
         <v>18</v>
       </c>
       <c r="I10" s="114"/>
+      <c r="K10" s="99" t="s">
+        <v>382</v>
+      </c>
+      <c r="L10" s="99" t="s">
+        <v>382</v>
+      </c>
+      <c r="M10" s="99" t="s">
+        <v>803</v>
+      </c>
+      <c r="N10" s="102"/>
+      <c r="O10" s="99" t="s">
+        <v>330</v>
+      </c>
+      <c r="P10" s="105" t="s">
+        <v>804</v>
+      </c>
+      <c r="Q10" s="110" t="s">
+        <v>394</v>
+      </c>
+      <c r="R10" s="111" t="s">
+        <v>18</v>
+      </c>
+      <c r="S10" s="114"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>

<commit_message>
fix(examples): name the zone 1 workbook channels after the DTR nodes
</commit_message>
<xml_diff>
--- a/examples/Model/Wind/IECA2015/Excel/Producer.xlsx
+++ b/examples/Model/Wind/IECA2015/Excel/Producer.xlsx
@@ -2342,7 +2342,7 @@
     <t>InternalNode1_BUS_Voltage</t>
   </si>
   <si>
-    <t>Wind_Turbine_GEN_VoltageInjTerminal</t>
+    <t>Wind_Turbine_GEN_VoltageNode2</t>
   </si>
   <si>
     <t>Wind_Turbine_GEN_ActivePowerSetpointPu</t>
@@ -2351,16 +2351,16 @@
     <t>Wind_Turbine_GEN_ReactivePowerSetpointPu</t>
   </si>
   <si>
-    <t>Wind_Turbine_GEN_ActivePowerControlledPu</t>
-  </si>
-  <si>
-    <t>Wind_Turbine_GEN_ReactivePowerControlledPu</t>
-  </si>
-  <si>
-    <t>Wind_Turbine_GEN_ActiveCurrentInjTerminal</t>
-  </si>
-  <si>
-    <t>Wind_Turbine_GEN_ReactiveCurrentInjTerminal</t>
+    <t>Wind_Turbine_GEN_ActivePowerControlledNode</t>
+  </si>
+  <si>
+    <t>Wind_Turbine_GEN_ReactivePowerControlledNode</t>
+  </si>
+  <si>
+    <t>Wind_Turbine_GEN_ActiveCurrentNode2</t>
+  </si>
+  <si>
+    <t>Wind_Turbine_GEN_ReactiveCurrentNode2</t>
   </si>
   <si>
     <t>../ReferenceCurves/Producer</t>

</xml_diff>